<commit_message>
test: update product and admin test cases
</commit_message>
<xml_diff>
--- a/test-cases/Ecommerce_Testing_TestCases.xlsx
+++ b/test-cases/Ecommerce_Testing_TestCases.xlsx
@@ -5,17 +5,19 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ecommerce-manual-testing\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D00FBAE-5098-40DC-A4D2-1F58511C6A27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D43CD6D-0537-490B-BEC6-46B0FE5BD580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{A63704CD-D83D-4C04-ADA8-4C9FC39B126E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{A63704CD-D83D-4C04-ADA8-4C9FC39B126E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sign Up" sheetId="2" r:id="rId1"/>
     <sheet name="Product" sheetId="3" r:id="rId2"/>
-    <sheet name="Sign In" sheetId="1" r:id="rId3"/>
+    <sheet name="Admin_Product" sheetId="4" r:id="rId3"/>
+    <sheet name="Admin_Category" sheetId="6" r:id="rId4"/>
+    <sheet name="Sign In" sheetId="1" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -27,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="228">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -247,9 +249,6 @@
     <t>1. Trên thanh địa chỉ trình duyệt, nhập URL: http://localhost:5173/admin/user 
 2. Nhấn Enter. 
 3. Quan sát kết quả hiển thị.</t>
-  </si>
-  <si>
-    <t>x</t>
   </si>
   <si>
     <t>• Hiển thị thông báo "Bạn không có quyền truy cập".
@@ -607,42 +606,455 @@
     <t>Kiểm tra tìm kiếm sản phẩm với từ khóa hợp lệ.</t>
   </si>
   <si>
-    <t>1. Nhập từ khóa "bông tai" vào ô tìm kiếm.
-2. Quan sát kết quả tìm kiếm.</t>
-  </si>
-  <si>
     <t>1. User đang ở trang chủ.
 2. Hệ thống có sản phẩm chứa từ khóa cần tìm.</t>
   </si>
   <si>
-    <t>Keyword: bông tai</t>
-  </si>
-  <si>
-    <t>• Hiển thị danh sách sản phẩm liên quan đến từ khóa "bông tai".
+    <t>TC_PRODUCT_003</t>
+  </si>
+  <si>
+    <t>1. User đang ở trang chủ.
+2. Hệ thống không có sản phẩm chứa từ khóa cần tìm.</t>
+  </si>
+  <si>
+    <t>Kiểm tra tìm kiếm với từ khóa không có sản phẩm phù hợp.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_004</t>
+  </si>
+  <si>
+    <t>1. User đang ở trang chủ.
+2. Menu Trang Sức có hiển thị danh sách category.</t>
+  </si>
+  <si>
+    <t>Kiểm tra hiển thị sản phẩm theo category.</t>
+  </si>
+  <si>
+    <t>1. Mở menu trang sức.
+2. Chọn category.
+3. Quan sát danh sách sản phẩm được hiển thị.</t>
+  </si>
+  <si>
+    <t>1. Nhập từ khóa vào ô tìm kiếm.
+2. Quan sát kết quả tìm kiếm.</t>
+  </si>
+  <si>
+    <t>• Hiển thị top 8 sản phẩm liên quan đến từ khóa cần tìm .
 • Các sản phẩm tìm được hiển thị thông tin như tên, hình ảnh và giá.
 • Không hiển thị sản phẩm không liên quan đến từ khóa tìm kiếm.
 • Không xuất hiện lỗi khi tải thông tin sản phẩm.</t>
   </si>
   <si>
-    <t>TC_PRODUCT_003</t>
-  </si>
-  <si>
-    <t>1. User đang ở trang chủ.
-2. Hệ thống không có sản phẩm chứa từ khóa cần tìm.</t>
-  </si>
-  <si>
-    <t>1. Nhập từ khóa "giày da" vào ô tìm kiếm.
-2. Quan sát kết quả tìm kiếm.</t>
-  </si>
-  <si>
-    <t>Keyword: giày da</t>
-  </si>
-  <si>
-    <t>• Hiển thị thông báo"Không tìm thấy sản phẩm phù hợp. Vui lòng thử từ khóa khác.".
+    <t>Keyword: giày da.</t>
+  </si>
+  <si>
+    <t>Keyword: bông tai.</t>
+  </si>
+  <si>
+    <t>Category: Nhẫn.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_005</t>
+  </si>
+  <si>
+    <t>Kiểm tra tìm kiếm với từ khóa có chứa khoảng trắng.</t>
+  </si>
+  <si>
+    <t>Keyword: " con heo ".</t>
+  </si>
+  <si>
+    <t>• Hiển thị top 8 sản phẩm liên quan đến từ khóa cần tìm bỏ qua khoảng trắng.
+• Các sản phẩm tìm được hiển thị thông tin như tên, hình ảnh và giá.
+• Không hiển thị sản phẩm không liên quan đến từ khóa tìm kiếm.
+• Không xuất hiện lỗi khi tải thông tin sản phẩm.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_006</t>
+  </si>
+  <si>
+    <t>Kiểm tra hiển thị của sản phẩm đã hết hàng.</t>
+  </si>
+  <si>
+    <t>1. User đang ở trang chi tiết sản phẩm.
+2. Sản phẩm có số lượng tồn kho = 0.</t>
+  </si>
+  <si>
+    <t>Product: một sản phẩm có stock = 0.</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_007</t>
+  </si>
+  <si>
+    <t>1. User đang ở trang chi tiết sản phẩm.
+2. Sản phẩm có số lượng tồn kho &gt; 0.</t>
+  </si>
+  <si>
+    <t>Product: một sản phẩm có stock &gt; 0.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Mở trang chi tiết của một sản phẩm còn hàng.
+2. Quan sát trạng thái sản phẩm.
+3. Quan sát các nút Mua ngay, Giỏ hàng, Gọi ngay.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Mở trang chi tiết của một sản phẩm hết hàng.
+2. Quan sát trạng thái sản phẩm.
+3. Quan sát các nút Mua ngay, Giỏ hàng, Gọi ngay.
+</t>
+  </si>
+  <si>
+    <t>• Hiển thị trạng thái Hết hàng.
+• Hiển thị thông báo sản phẩm hiện không có sẵn.
+• Các nút mua hàng như Gọi ngay, Mua ngay và Giỏ hàng bị disable/không cho thao tác.
+• User không thể tạo giao dịch mua đối với sản phẩm hết hàng.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+• User được chuyển đến trang danh sách sản phẩm chỉ có category đã chọn.
+• Hiển thị đúng danh sách sản phẩm thuộc category đã chọn.
+• Không xuất hiện lỗi khi tải thông tin sản phẩm.
+• Không hiển thị sản phẩm thuộc category khác.</t>
+  </si>
+  <si>
+    <t>TC_ADMIN_PRODUCT_001</t>
+  </si>
+  <si>
+    <t>Tạo sản phẩm mới với dữ liệu hợp lệ</t>
+  </si>
+  <si>
+    <t>1. User có role Admin hoặc Staff có quyền quản lý sản phẩm.
+2. User đã đăng nhập thành công.
+3. User đang ở trang quản lý sản phẩm.</t>
+  </si>
+  <si>
+    <t>• Tạo sản phẩm thành công.
+• Hiển thị thông báo tạo sản phẩm thành công.
+• Sản phẩm mới xuất hiện trong danh sách quản lý sản phẩm.
+• Thông tin sản phẩm được lưu đúng với dữ liệu đã nhập.
+• Sản phẩm có thể được tìm thấy/hiển thị ở phía Customer nếu trạng thái cho phép bán.</t>
+  </si>
+  <si>
+    <t>TC_ADMIN_PRODUCT_002</t>
+  </si>
+  <si>
+    <t>Tạo sản phẩm khi bỏ trống một field bắt buộc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Không tạo sản phẩm.
+ • Hiển thị thông báo Thiếu thông tin.
+ • Hiển thị nội dung Vui lòng điền đầy đủ các trường và chọn ít nhất 1 ảnh.
+ • User vẫn ở trang thêm sản phẩm.
+ • Không có sản phẩm mới được tạo.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Không tạo sản phẩm.
+ • Hiển thị thông báo Thiếu thông tin.
+ • Hiển thị nội dung "Vui lòng điền đầy đủ các trường và chọn ít nhất 1 ảnh".
+ • User vẫn ở trang thêm sản phẩm.
+ • Không có sản phẩm mới được tạo.  </t>
+  </si>
+  <si>
+    <t>TC_ADMIN_PRODUCT_003</t>
+  </si>
+  <si>
+    <t>Tạo category mới với dữ liệu hợp lệ</t>
+  </si>
+  <si>
+    <t>1. Nhấn nút "Add New Category".
+2. Nhập Category Name.
+3. Nhập Description.
+4. Nhấn nút "Add Category".
+5. Quan sát kết quả.</t>
+  </si>
+  <si>
+    <t>• Category Name: Test Category.
+• Description: TestCategory.</t>
+  </si>
+  <si>
+    <t>• Tạo category thành công.
+• Hiển thị thông báo tạo category thành công.
+• Category mới xuất hiện trong danh sách category.
+• Category Name và Description được lưu đúng với dữ liệu đã nhập.
+• Category mới có thể được chọn trong trường Danh mục khi Admin/Staff tạo hoặc chỉnh sửa sản phẩm.</t>
+  </si>
+  <si>
+    <t>TC_ADMIN_PRODUCT_004</t>
+  </si>
+  <si>
+    <t>Tạo category khi bỏ trống Category Name.</t>
+  </si>
+  <si>
+    <t>• Category Name:  [empty].
+• Description: TestCategory.</t>
+  </si>
+  <si>
+    <t>• Tạo category thành công.
+• Hiển thị thông báo tạo category thành công.
+• Category mới xuất hiện trong danh sách category.
+• Category Name là khoảng trắng và Description được lưu đúng với dữ liệu đã nhập.
+• Category mới có thể được chọn trong trường Danh mục khi Admin/Staff tạo hoặc chỉnh sửa sản phẩm.</t>
+  </si>
+  <si>
+    <t>TC_ADMIN_PRODUCT_005</t>
+  </si>
+  <si>
+    <t>1. Nhấn nút "Add New Category".
+2. Để trống Category Name.
+3. Nhập Description.
+4. Nhấn nút "Add Category".
+5. Quan sát kết quả.</t>
+  </si>
+  <si>
+    <t>1. Nhấn nút "Add New Category".
+2. Nhập Category Name.
+3. Để trống Description.
+4. Nhấn nút "Add Category".
+5. Quan sát kết quả.</t>
+  </si>
+  <si>
+    <t>• Category Name: Test Category.
+• Description: [empty].</t>
+  </si>
+  <si>
+    <t>Tạo category khi bỏ trống Description</t>
+  </si>
+  <si>
+    <t>TC_ADMIN_CATEGORY_001</t>
+  </si>
+  <si>
+    <t>TC_ADMIN_CATEGORY_002</t>
+  </si>
+  <si>
+    <t>TC_ADMIN_CATEGORY_003</t>
+  </si>
+  <si>
+    <t>Chỉnh sửa thông tin sản phẩm với dữ liệu hợp lệ</t>
+  </si>
+  <si>
+    <t>1. Nhấn nút "Edit" ở sản phẩm cần chỉnh sửa.
+2. Nhập hợp lệ các thông tin cần chỉnh sửa.
+3. Nhấn nút "Update Product".
+4. Quan sát kết quả.</t>
+  </si>
+  <si>
+    <t>• Hiển thị thông báo cập nhật sản phẩm thành công.
+• Thông tin sản phẩm được lưu đúng với dữ liệu đã chỉnh sửa.
+• Sản phẩm có thể được tìm thấy/hiển thị ở phía Customer nếu trạng thái cho phép bán.</t>
+  </si>
+  <si>
+    <t>1. Nhấn nút "Edit" ở sản phẩm cần chỉnh sửa.
+2. Giảm "Quantity" sản phẩm về 0.
+3. Nhấn nút "Update Product".
+4. Quan sát kết quả.</t>
+  </si>
+  <si>
+    <t>Cập nhật Quantity từ &gt;0 về 0 và kiểm tra phía Customer hiển thị Hết hàng</t>
+  </si>
+  <si>
+    <t>• Product Name: Test Product 001.
+• Description:Test Product 001.
+• Price: 500000
+• Quantity: 1
+• Category: Nhẫn
+• Images: file ảnh hợp lệ</t>
+  </si>
+  <si>
+    <t>1. Nhấn nút "Add New Product".
+2. Nhập đầy đủ các thông tin hợp lệ của sản phẩm.
+3. Nhập Price bán hợp lệ.
+4. Nhập Quantity tồn kho hợp lệ.
+5. Chọn Category sản phẩm.
+6. Thêm Images sản phẩm.
+7. Nhấn nút "Add Product".
+8. Kiểm tra sản phẩm trong danh sách quản lý.
+9. Truy cập phía Customer và mở sản phẩm vừa tạo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Nhấn nút "Add New Product".
+2. Nhập hợp lệ các field còn lại.
+3. Để trống một field bắt buộc cần kiểm tra.
+4. Nhấn nút "Add Product".
+5. Quan sát kết quả.
+</t>
+  </si>
+  <si>
+    <t>• User được chuyển đến trang danh sách sản phẩm chỉ có category đã chọn.
+• Hiển thị đúng danh sách sản phẩm thuộc category đã chọn.
+• Không xuất hiện lỗi khi tải thông tin sản phẩm.
+• Không hiển thị sản phẩm thuộc category khác.</t>
+  </si>
+  <si>
+    <t>• Cập nhật số lượng tồn kho của sản phẩm từ &gt; 0 về 0 thành công.
+• Tại trang quản lý sản phẩm, stock của sản phẩm được hiển thị là 0.
+• Khi Customer mở trang chi tiết sản phẩm, hệ thống hiển thị trạng thái Hết hàng.
+• Hiển thị thông báo sản phẩm hiện không có sẵn.
+• Các chức năng mua hàng như Mua ngay và Giỏ hàng bị disable/không thể thao tác.
+• Customer không thể thêm sản phẩm hết hàng vào giỏ hàng hoặc thực hiện mua sản phẩm</t>
+  </si>
+  <si>
+    <t>• Tên sản phẩm: TestProduct 001.
+• Description:Test Product 001.
+• Price: 500000
+• Quantity: 100
+• Category: Nhẫn
+• Images: file ảnh hợp lệ</t>
+  </si>
+  <si>
+    <t>• Cập nhật số lượng tồn kho của sản phẩm từ 0 lên giá trị &gt; 0 thành công.
+• Tại trang quản lý sản phẩm, stock hiển thị đúng giá trị mới.
+• Khi Customer mở trang chi tiết sản phẩm, hệ thống hiển thị trạng thái Còn hàng.
+• Hiển thị đúng giá sản phẩm và số lượng còn lại.
+• Các nút Mua ngay và Giỏ hàng hoạt động bình thường.
+• Customer có thể thêm sản phẩm vào giỏ hàng hoặc thực hiện mua sản phẩm.</t>
+  </si>
+  <si>
+    <t>Cập nhật stock từ 0 lên &gt;0 và kiểm tra phía Customer hiển thị Còn hàng</t>
+  </si>
+  <si>
+    <t>TC_ADMIN_PRODUCT_006</t>
+  </si>
+  <si>
+    <t>Kiểm tra tắt trạng thái bán của sản phẩm và xác nhận Customer không còn nhìn thấy sản phẩm.</t>
+  </si>
+  <si>
+    <t>1. User có role Admin hoặc Staff có quyền quản lý sản phẩm.
+2. Sản phẩm đang ở trạng thái Đang mở bán
+3. Sản phẩm đang hiển thị ở phía Customer.</t>
+  </si>
+  <si>
+    <t>1. Truy cập trang quản lý sản phẩm.
+2. Tìm sản phẩm cần kiểm tra.
+3. Tắt trạng thái Đang mở bán.
+4. Quan sát trạng thái sản phẩm ở trang Admin.
+5. Truy cập phía Customer.
+6. Tìm kiếm sản phẩm bằng tên hoặc truy cập category chứa sản phẩm.
+7. Quan sát kết quả.</t>
+  </si>
+  <si>
+    <t>• Product: Test Product 001.
+• Status trước: Đang mở bán.
+• Status sau: Tắt bán</t>
+  </si>
+  <si>
+    <t>TC_PRODUCT_008</t>
+  </si>
+  <si>
+    <t>Kiểm tra truy cập trực tiếp URL của sản phẩm đã tắt bán.</t>
+  </si>
+  <si>
+    <t>1. Admin đã tắt trạng thái bán của sản phẩm.
+2. Có URL của sản phẩm trước khi bị tắt.</t>
+  </si>
+  <si>
+    <t>1. Truy cập phía Customer.
+2. Nhập trực tiếp URL của sản phẩm đã tắt bán vào thanh địa chỉ trình duyệt.
+3. Nhấn Enter.
+4. Quan sát kết quả.</t>
+  </si>
+  <si>
+    <t>Product: Test Product 001
+Status: Tắt bán
+URL:http://localhost:5173/product/&lt;product-id&gt;</t>
+  </si>
+  <si>
+    <t>• Customer vẫn truy cập được trực tiếp URL của sản phẩm đã tắt bán.
+• Trang Product Detail vẫn hiển thị thông tin sản phẩm.</t>
+  </si>
+  <si>
+    <t>• Hiển thị thông báo “Sản phẩm không tồn tại” và đếm ngược 3 giây.
+• Sau 3 giây, hệ thống tự động chuyển Customer về Trang chủ.
+• Không hiển thị thông tin chi tiết của sản phẩm đã tắt bán.
+• Customer không thể thực hiện thao tác Mua ngay hoặc Thêm vào giỏ hàng.</t>
+  </si>
+  <si>
+    <t>TC_ADMIN_CATEGORY_004</t>
+  </si>
+  <si>
+    <t>Kiểm tra chỉnh sửa Category với dữ liệu hợp lệ.</t>
+  </si>
+  <si>
+    <t>1. User có role Admin hoặc Staff có quyền quản lý category.
+2. User đã đăng nhập thành công.
+3. User đang ở trang quản lý category.</t>
+  </si>
+  <si>
+    <t>1. Chọn category muốn chỉnh sửa.
+2. Nhấn nút "Edit".
+3. Nhập thông tin cần sửa hợp lệ.
+4. Nhấn nút "Update Category".
+5. Quan sát kết quả.</t>
+  </si>
+  <si>
+    <t>• Category Name: Test Category1234.
+• Description: TestCategory.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Không tạo category.
+ • Hiển thị thông báo Thiếu thông tin.
+ • Hiển thị nội dung Vui lòng nhập Category Name.
+ • User vẫn ở trang Add New Category.
+ • Không có category mới được tạo.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Không tạo category.
+ • Hiển thị thông báo Thiếu thông tin.
+ • Hiển thị nội dung Vui lòng nhập Description.
+ • User vẫn ở trang Add New Category.
+ • Không có category mới được tạo.  </t>
+  </si>
+  <si>
+    <t>• Hiển thị thông báo cập nhật category thành công.
+• Category Name và Description được lưu đúng với dữ liệu đã chỉnh sửa.
+• Category sau khi cập nhật có thể được chọn trong trường Danh mục khi Admin/Staff tạo hoặc chỉnh sửa sản phẩm.</t>
+  </si>
+  <si>
+    <t>• Hiển thị thông báo"Không tìm thấy sản phẩm phù hợp. Vui lòng thử từ khóa khác".
 • Không hiển thị sản phẩm không liên quan đến từ khóa tìm kiếm.</t>
   </si>
   <si>
-    <t>Kiểm tra tìm kiếm với từ khóa không có sản phẩm phù hợp.</t>
+    <t>Kiểm tra hiển thị của sản phẩm còn hàng.</t>
+  </si>
+  <si>
+    <t>• Hiển thị trạng thái còn hàng.
+• Hiển thị đúng giá sản phẩm và số lượng còn lại.
+• Các nút mua hàng như Mua ngay và Giỏ hàng vẫn hoạt động bình thường.
+• User có thể thêm sản phẩm vào giỏ hàng.</t>
+  </si>
+  <si>
+    <t>• Iteration 1: Product Name = [empty]
+• Iteration 2: Description = [empty]
+• Iteration 3: Price = [empty]
+• Iteration 4: Quantity = [empty]
+• Iteration 5: Category = [empty]
+• Iteration 6: Images = [empty]</t>
+  </si>
+  <si>
+    <t>• Product Name: Test_Product 002.
+• Description:Test Product 001.
+• Price: 500000
+• Quantity: 1
+• Category: Nhẫn
+• Images: file ảnh hợp lệ</t>
+  </si>
+  <si>
+    <t>1. Nhấn nút "Edit" ở sản phẩm cần chỉnh sửa.
+2. Giảm "Quantity" sản phẩm từ 0 lên 100.
+3. Nhấn nút "Update Product".
+4. Quan sát kết quả.</t>
+  </si>
+  <si>
+    <t>• Tên sản phẩm: Test_Product 002.
+• Description:Test Product 001.
+• Price: 500000
+• Quantity: 0
+• Category: Nhẫn
+• Images: file ảnh hợp lệ</t>
+  </si>
+  <si>
+    <t>• Sản phẩm vẫn còn trong danh sách quản lý của Admin với trạng thái đang mở bán tắt.
+• Sản phẩm không còn xuất hiện trong danh sách sản phẩm phía Customer.
+• Customer không tìm thấy sản phẩm bằng chức năng Search.</t>
   </si>
 </sst>
 </file>
@@ -677,7 +1089,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -687,6 +1099,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF7575"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -718,7 +1136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -754,6 +1172,34 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1128,7 +1574,7 @@
         <v>33</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>30</v>
@@ -1140,91 +1586,91 @@
         <v>32</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H2" s="5" t="s">
         <v>29</v>
       </c>
       <c r="I2" s="3"/>
     </row>
-    <row r="3" spans="1:16" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
         <v>41</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D3" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="E3" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>68</v>
-      </c>
       <c r="G3" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>29</v>
       </c>
       <c r="I3" s="3"/>
     </row>
-    <row r="4" spans="1:16" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="D4" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>70</v>
-      </c>
       <c r="E4" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>29</v>
       </c>
       <c r="I4" s="3"/>
     </row>
-    <row r="5" spans="1:16" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H5" s="5" t="s">
         <v>29</v>
@@ -1233,79 +1679,79 @@
     </row>
     <row r="6" spans="1:16" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>29</v>
       </c>
       <c r="I6" s="3"/>
     </row>
-    <row r="7" spans="1:16" ht="109.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:16" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D7" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="E7" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="E7" s="8" t="s">
-        <v>91</v>
-      </c>
       <c r="F7" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>29</v>
       </c>
       <c r="I7" s="3"/>
     </row>
-    <row r="8" spans="1:16" ht="124.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E8" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="F8" s="4" t="s">
-        <v>81</v>
-      </c>
       <c r="G8" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>29</v>
@@ -1314,25 +1760,25 @@
     </row>
     <row r="9" spans="1:16" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="E9" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="E9" s="8" t="s">
+      <c r="F9" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="F9" s="4" t="s">
-        <v>94</v>
-      </c>
       <c r="G9" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>29</v>
@@ -1341,106 +1787,106 @@
     </row>
     <row r="10" spans="1:16" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>96</v>
-      </c>
       <c r="C10" s="11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D10" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="E10" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="E10" s="11" t="s">
-        <v>126</v>
-      </c>
       <c r="F10" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="H10" s="12" t="s">
         <v>99</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="H10" s="12" t="s">
-        <v>100</v>
       </c>
       <c r="I10" s="3"/>
     </row>
     <row r="11" spans="1:16" ht="93.6" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="B11" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="B11" s="10" t="s">
-        <v>102</v>
-      </c>
       <c r="C11" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D11" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="E11" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="F11" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="F11" s="10" t="s">
-        <v>109</v>
-      </c>
       <c r="G11" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H11" s="12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I11" s="3"/>
     </row>
     <row r="12" spans="1:16" ht="109.2" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="C12" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="D12" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="C12" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="D12" s="8" t="s">
+      <c r="E12" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="E12" s="4" t="s">
-        <v>113</v>
-      </c>
       <c r="F12" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H12" s="5" t="s">
         <v>29</v>
       </c>
       <c r="I12" s="3"/>
     </row>
-    <row r="13" spans="1:16" ht="171.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" ht="124.8" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E13" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="E13" s="8" t="s">
+      <c r="F13" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="F13" s="8" t="s">
-        <v>118</v>
-      </c>
       <c r="G13" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H13" s="5" t="s">
         <v>29</v>
@@ -1449,23 +1895,23 @@
     </row>
     <row r="14" spans="1:16" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>120</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="C14" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="D14" s="8" t="s">
         <v>121</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>122</v>
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H14" s="5" t="s">
         <v>29</v>
@@ -2367,8 +2813,8 @@
     <col min="2" max="2" width="26.6640625" style="2" customWidth="1"/>
     <col min="3" max="3" width="26" style="2" customWidth="1"/>
     <col min="4" max="4" width="35.77734375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="24.44140625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="34" style="2" customWidth="1"/>
+    <col min="5" max="5" width="39.77734375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="39.33203125" style="2" customWidth="1"/>
     <col min="7" max="7" width="31.88671875" style="2" customWidth="1"/>
     <col min="8" max="8" width="11.109375" style="2" customWidth="1"/>
     <col min="9" max="9" width="11.21875" style="2" customWidth="1"/>
@@ -2406,25 +2852,25 @@
     </row>
     <row r="2" spans="1:9" ht="112.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="F2" s="4" t="s">
-        <v>131</v>
-      </c>
       <c r="G2" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H2" s="5" t="s">
         <v>29</v>
@@ -2433,25 +2879,25 @@
     </row>
     <row r="3" spans="1:9" ht="124.8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B3" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>136</v>
-      </c>
       <c r="D3" s="4" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>29</v>
@@ -2460,84 +2906,164 @@
     </row>
     <row r="4" spans="1:9" ht="78" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>142</v>
-      </c>
       <c r="F4" s="4" t="s">
-        <v>143</v>
+        <v>220</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>143</v>
+        <v>220</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>29</v>
       </c>
       <c r="I4" s="3"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
+    <row r="5" spans="1:9" ht="140.4" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>29</v>
+      </c>
       <c r="I5" s="3"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
+    <row r="6" spans="1:9" ht="156" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>29</v>
+      </c>
       <c r="I6" s="3"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
+    <row r="7" spans="1:9" ht="124.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>29</v>
+      </c>
       <c r="I7" s="3"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
+    <row r="8" spans="1:9" ht="124.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>29</v>
+      </c>
       <c r="I8" s="3"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
+    <row r="9" spans="1:9" ht="124.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="14" t="s">
+        <v>205</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>211</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>99</v>
+      </c>
       <c r="I9" s="3"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -2664,12 +3190,436 @@
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21D6234B-C587-4229-A515-D800C628ED15}">
+  <dimension ref="A1:I22"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="27.5546875" style="6" customWidth="1"/>
+    <col min="2" max="2" width="26.6640625" style="6" customWidth="1"/>
+    <col min="3" max="3" width="32" style="6" customWidth="1"/>
+    <col min="4" max="4" width="41.109375" style="6" customWidth="1"/>
+    <col min="5" max="5" width="37.33203125" style="6" customWidth="1"/>
+    <col min="6" max="6" width="36.77734375" style="6" customWidth="1"/>
+    <col min="7" max="7" width="36.88671875" style="6" customWidth="1"/>
+    <col min="8" max="8" width="11.6640625" style="6" customWidth="1"/>
+    <col min="9" max="9" width="13.33203125" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="184.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I2" s="3"/>
+    </row>
+    <row r="3" spans="1:9" ht="109.2" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I3" s="3"/>
+    </row>
+    <row r="4" spans="1:9" ht="109.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" s="3"/>
+    </row>
+    <row r="5" spans="1:9" ht="234" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="202.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="140.4" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H8" s="13"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H9" s="13"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H10" s="13"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H11" s="13"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H12" s="13"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H13" s="13"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H14" s="13"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H15" s="13"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H16" s="13"/>
+    </row>
+    <row r="17" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H17" s="13"/>
+    </row>
+    <row r="18" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H18" s="13"/>
+    </row>
+    <row r="19" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H19" s="13"/>
+    </row>
+    <row r="20" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H20" s="13"/>
+    </row>
+    <row r="21" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H21" s="13"/>
+    </row>
+    <row r="22" spans="8:8" x14ac:dyDescent="0.3">
+      <c r="H22" s="13"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CABB5BA-899C-47CE-A01D-B6742958302D}">
+  <dimension ref="A1:Q5"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="30.109375" style="18" customWidth="1"/>
+    <col min="2" max="2" width="22" style="18" customWidth="1"/>
+    <col min="3" max="3" width="28.6640625" style="18" customWidth="1"/>
+    <col min="4" max="4" width="32.77734375" style="18" customWidth="1"/>
+    <col min="5" max="5" width="29.6640625" style="18" customWidth="1"/>
+    <col min="6" max="6" width="34.5546875" style="18" customWidth="1"/>
+    <col min="7" max="7" width="35.44140625" style="18" customWidth="1"/>
+    <col min="8" max="8" width="8.88671875" style="18"/>
+    <col min="9" max="9" width="16.44140625" style="18" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="18"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A1" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="16" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="21" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" ht="171.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>214</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>172</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>173</v>
+      </c>
+      <c r="F2" s="19" t="s">
+        <v>174</v>
+      </c>
+      <c r="G2" s="19" t="s">
+        <v>174</v>
+      </c>
+      <c r="H2" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="I2" s="16"/>
+      <c r="J2" s="16"/>
+      <c r="K2" s="16"/>
+      <c r="L2" s="16"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
+      <c r="P2" s="16"/>
+      <c r="Q2" s="17"/>
+    </row>
+    <row r="3" spans="1:17" ht="226.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" ht="171.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="140.4" x14ac:dyDescent="0.3">
+      <c r="A5" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>214</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>215</v>
+      </c>
+      <c r="E5" s="19" t="s">
+        <v>216</v>
+      </c>
+      <c r="F5" s="19" t="s">
+        <v>219</v>
+      </c>
+      <c r="G5" s="19" t="s">
+        <v>219</v>
+      </c>
+      <c r="H5" s="20" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1BAC9A9-C36E-4351-8CDF-6213253BAC2A}">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.109375" style="2" customWidth="1"/>
@@ -2776,7 +3726,7 @@
         <v>13</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>27</v>
@@ -2796,10 +3746,10 @@
         <v>37</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>28</v>
@@ -2822,10 +3772,10 @@
         <v>38</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>18</v>
@@ -2877,7 +3827,7 @@
         <v>48</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>22</v>
@@ -2903,7 +3853,7 @@
         <v>47</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>49</v>
@@ -2929,7 +3879,7 @@
         <v>46</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>50</v>
@@ -2955,7 +3905,7 @@
         <v>53</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>58</v>
@@ -2964,10 +3914,10 @@
         <v>54</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>29</v>
@@ -2981,7 +3931,7 @@
         <v>56</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>58</v>
@@ -2990,19 +3940,17 @@
         <v>57</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H12" s="5" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E16" s="2" t="s">
-        <v>59</v>
-      </c>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B13" s="22"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>